<commit_message>
Fix failing unit tests for xlsx import
</commit_message>
<xml_diff>
--- a/tests/data/rdi_correct.xlsx
+++ b/tests/data/rdi_correct.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="103">
   <si>
     <t xml:space="preserve">household_id</t>
   </si>
@@ -310,6 +310,9 @@
   </si>
   <si>
     <t xml:space="preserve">pp_country_i_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pp_gender_i_c</t>
   </si>
   <si>
     <t xml:space="preserve">Collector ForJanIndex_3</t>
@@ -337,14 +340,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
     <numFmt numFmtId="166" formatCode="@"/>
-    <numFmt numFmtId="167" formatCode="General"/>
-    <numFmt numFmtId="168" formatCode="m/d/yyyy"/>
-    <numFmt numFmtId="169" formatCode="0"/>
-    <numFmt numFmtId="170" formatCode="d/m/yyyy\ hh:mm:ss"/>
+    <numFmt numFmtId="167" formatCode="m/d/yyyy"/>
+    <numFmt numFmtId="168" formatCode="0"/>
+    <numFmt numFmtId="169" formatCode="d/m/yyyy\ hh:mm:ss"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -478,15 +480,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -494,7 +492,11 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="169" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -538,9 +540,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>97560</xdr:colOff>
+      <xdr:colOff>97200</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>94680</xdr:rowOff>
+      <xdr:rowOff>94320</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -554,11 +556,12 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="17452440" y="380880"/>
-          <a:ext cx="97560" cy="94680"/>
+          <a:ext cx="97200" cy="94320"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:noFill/>
         <a:ln w="0">
           <a:noFill/>
         </a:ln>
@@ -575,9 +578,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>97920</xdr:colOff>
+      <xdr:colOff>97560</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>95040</xdr:rowOff>
+      <xdr:rowOff>94680</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -591,11 +594,12 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10877400" y="380880"/>
-          <a:ext cx="97920" cy="95040"/>
+          <a:ext cx="97560" cy="94680"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:noFill/>
         <a:ln w="0">
           <a:noFill/>
         </a:ln>
@@ -787,7 +791,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:O4"/>
-  <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9.63"/>
@@ -801,7 +805,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="19.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="18.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="1" width="19.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16381" style="0" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16381" style="1" width="10.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -920,7 +924,7 @@
       <c r="A4" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B4" s="7" t="b">
+      <c r="B4" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -978,7 +982,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:P13"/>
-  <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.82"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.97"/>
@@ -995,8 +999,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="21.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="1" width="19.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="11.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16383" min="16383" style="0" width="10.16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16383" style="1" width="10.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1088,10 +1091,10 @@
       <c r="I3" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J3" s="8" t="n">
+      <c r="J3" s="7" t="n">
         <v>28558</v>
       </c>
-      <c r="K3" s="9" t="n">
+      <c r="K3" s="8" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1133,10 +1136,10 @@
       <c r="I4" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J4" s="8" t="n">
+      <c r="J4" s="7" t="n">
         <v>43298</v>
       </c>
-      <c r="K4" s="9" t="n">
+      <c r="K4" s="8" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1178,10 +1181,10 @@
       <c r="I5" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J5" s="8" t="n">
+      <c r="J5" s="7" t="n">
         <v>24971</v>
       </c>
-      <c r="K5" s="9" t="n">
+      <c r="K5" s="8" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1220,10 +1223,10 @@
       <c r="I6" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J6" s="8" t="n">
+      <c r="J6" s="7" t="n">
         <v>24092</v>
       </c>
-      <c r="K6" s="9" t="n">
+      <c r="K6" s="8" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1265,10 +1268,10 @@
       <c r="I7" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J7" s="8" t="n">
+      <c r="J7" s="7" t="n">
         <v>34615</v>
       </c>
-      <c r="K7" s="9" t="n">
+      <c r="K7" s="8" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1307,10 +1310,10 @@
       <c r="I8" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J8" s="8" t="n">
+      <c r="J8" s="7" t="n">
         <v>25778</v>
       </c>
-      <c r="K8" s="7" t="b">
+      <c r="K8" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1349,10 +1352,10 @@
       <c r="I9" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J9" s="8" t="n">
+      <c r="J9" s="7" t="n">
         <v>31934</v>
       </c>
-      <c r="K9" s="7" t="b">
+      <c r="K9" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1391,10 +1394,10 @@
       <c r="I10" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J10" s="8" t="n">
+      <c r="J10" s="7" t="n">
         <v>23346</v>
       </c>
-      <c r="K10" s="7" t="b">
+      <c r="K10" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1412,7 +1415,7 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J12" s="8"/>
+      <c r="J12" s="7"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="n">
@@ -1440,10 +1443,10 @@
       <c r="I13" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J13" s="8" t="n">
+      <c r="J13" s="7" t="n">
         <v>42889</v>
       </c>
-      <c r="K13" s="7" t="b">
+      <c r="K13" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1475,8 +1478,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="13.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30.18"/>
@@ -1484,6 +1487,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="21.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="17.64"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1505,85 +1509,100 @@
       <c r="F1" s="6" t="s">
         <v>94</v>
       </c>
+      <c r="G1" s="6" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="n">
+      <c r="A2" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B2" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="C2" s="12" t="n">
+      <c r="B2" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="C2" s="11" t="n">
         <v>37125</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
+      </c>
+      <c r="G2" s="12" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="10" t="n">
+      <c r="A3" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="C3" s="11" t="n">
+        <v>40777</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="F3" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="C3" s="12" t="n">
-        <v>40777</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>98</v>
+      <c r="G3" s="12" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="n">
+      <c r="A4" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="C4" s="12" t="n">
+      <c r="B4" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="C4" s="11" t="n">
         <v>33472</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="n">
+      <c r="A5" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="C5" s="12" t="n">
+      <c r="B5" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" s="11" t="n">
         <v>36760</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix fail if alien check Fix failing unit tests
</commit_message>
<xml_diff>
--- a/tests/data/rdi_correct.xlsx
+++ b/tests/data/rdi_correct.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Households" sheetId="1" state="visible" r:id="rId3"/>
@@ -63,13 +63,13 @@
     <t xml:space="preserve">consent_sharing_h_c</t>
   </si>
   <si>
-    <t xml:space="preserve">head_of_household_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">primary_collector_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">alternate_collector_id</t>
+    <t xml:space="preserve">head_of_household</t>
+  </si>
+  <si>
+    <t xml:space="preserve">primary_collector</t>
+  </si>
+  <si>
+    <t xml:space="preserve">alternate_collector</t>
   </si>
   <si>
     <t xml:space="preserve">AFG</t>
@@ -540,9 +540,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>97200</xdr:colOff>
+      <xdr:colOff>96840</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>94320</xdr:rowOff>
+      <xdr:rowOff>93960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -556,7 +556,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="17452440" y="380880"/>
-          <a:ext cx="97200" cy="94320"/>
+          <a:ext cx="96840" cy="93960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -578,9 +578,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>97560</xdr:colOff>
+      <xdr:colOff>97200</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>94680</xdr:rowOff>
+      <xdr:rowOff>94320</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -594,7 +594,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10877400" y="380880"/>
-          <a:ext cx="97560" cy="94680"/>
+          <a:ext cx="97200" cy="94320"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1487,7 +1487,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="21.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14.01"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="17.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="17.64"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
chg ! Aurora import (#269)
* chg ! Aurora import

* add ! save Aurora watermark

* tests

* drop versioning script for program Nigeria measles rubella campaign
</commit_message>
<xml_diff>
--- a/tests/data/rdi_correct.xlsx
+++ b/tests/data/rdi_correct.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="104">
   <si>
     <t xml:space="preserve">household_id</t>
   </si>
@@ -313,6 +313,9 @@
   </si>
   <si>
     <t xml:space="preserve">pp_gender_i_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pp_estimated_birth_date</t>
   </si>
   <si>
     <t xml:space="preserve">Collector ForJanIndex_3</t>
@@ -340,13 +343,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
     <numFmt numFmtId="166" formatCode="@"/>
-    <numFmt numFmtId="167" formatCode="m/d/yyyy"/>
-    <numFmt numFmtId="168" formatCode="0"/>
-    <numFmt numFmtId="169" formatCode="d/m/yyyy\ hh:mm:ss"/>
+    <numFmt numFmtId="167" formatCode="General"/>
+    <numFmt numFmtId="168" formatCode="m/d/yyyy"/>
+    <numFmt numFmtId="169" formatCode="0"/>
+    <numFmt numFmtId="170" formatCode="d/m/yyyy\ hh:mm:ss"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -447,7 +451,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -480,11 +484,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -492,12 +504,16 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="170" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -540,9 +556,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>97200</xdr:colOff>
+      <xdr:colOff>96120</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>94320</xdr:rowOff>
+      <xdr:rowOff>93240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -556,12 +572,11 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="17452440" y="380880"/>
-          <a:ext cx="97200" cy="94320"/>
+          <a:ext cx="96120" cy="93240"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
         <a:ln w="0">
           <a:noFill/>
         </a:ln>
@@ -578,9 +593,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>97560</xdr:colOff>
+      <xdr:colOff>96480</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>94680</xdr:rowOff>
+      <xdr:rowOff>93600</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -594,12 +609,11 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10877400" y="380880"/>
-          <a:ext cx="97560" cy="94680"/>
+          <a:ext cx="96480" cy="93600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
         <a:ln w="0">
           <a:noFill/>
         </a:ln>
@@ -791,7 +805,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:O4"/>
-  <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9.63"/>
@@ -924,7 +938,7 @@
       <c r="A4" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B4" s="1" t="b">
+      <c r="B4" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -982,7 +996,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:P13"/>
-  <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.82"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.97"/>
@@ -1091,10 +1105,10 @@
       <c r="I3" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J3" s="7" t="n">
+      <c r="J3" s="8" t="n">
         <v>28558</v>
       </c>
-      <c r="K3" s="8" t="n">
+      <c r="K3" s="9" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1136,10 +1150,10 @@
       <c r="I4" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J4" s="7" t="n">
+      <c r="J4" s="8" t="n">
         <v>43298</v>
       </c>
-      <c r="K4" s="8" t="n">
+      <c r="K4" s="9" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1181,10 +1195,10 @@
       <c r="I5" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J5" s="7" t="n">
+      <c r="J5" s="8" t="n">
         <v>24971</v>
       </c>
-      <c r="K5" s="8" t="n">
+      <c r="K5" s="9" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1223,10 +1237,10 @@
       <c r="I6" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J6" s="7" t="n">
+      <c r="J6" s="8" t="n">
         <v>24092</v>
       </c>
-      <c r="K6" s="8" t="n">
+      <c r="K6" s="9" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1268,10 +1282,10 @@
       <c r="I7" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J7" s="7" t="n">
+      <c r="J7" s="8" t="n">
         <v>34615</v>
       </c>
-      <c r="K7" s="8" t="n">
+      <c r="K7" s="9" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1310,10 +1324,10 @@
       <c r="I8" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J8" s="7" t="n">
+      <c r="J8" s="8" t="n">
         <v>25778</v>
       </c>
-      <c r="K8" s="1" t="b">
+      <c r="K8" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1352,10 +1366,10 @@
       <c r="I9" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J9" s="7" t="n">
+      <c r="J9" s="8" t="n">
         <v>31934</v>
       </c>
-      <c r="K9" s="1" t="b">
+      <c r="K9" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1394,10 +1408,10 @@
       <c r="I10" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J10" s="7" t="n">
+      <c r="J10" s="8" t="n">
         <v>23346</v>
       </c>
-      <c r="K10" s="1" t="b">
+      <c r="K10" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1415,7 +1429,7 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J12" s="7"/>
+      <c r="J12" s="8"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="n">
@@ -1443,10 +1457,10 @@
       <c r="I13" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J13" s="7" t="n">
+      <c r="J13" s="8" t="n">
         <v>42889</v>
       </c>
-      <c r="K13" s="1" t="b">
+      <c r="K13" s="7" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1478,8 +1492,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="13.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30.18"/>
@@ -1487,7 +1501,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="21.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14.01"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="17.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="17.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="22.2"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1512,97 +1527,116 @@
       <c r="G1" s="6" t="s">
         <v>95</v>
       </c>
+      <c r="H1" s="10" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="n">
+      <c r="A2" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="B2" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="C2" s="11" t="n">
+      <c r="B2" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="C2" s="13" t="n">
         <v>37125</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="G2" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="G2" s="14" t="s">
         <v>52</v>
+      </c>
+      <c r="H2" s="15" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="9" t="n">
+      <c r="A3" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="C3" s="13" t="n">
+        <v>40777</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="F3" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="C3" s="11" t="n">
-        <v>40777</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="G3" s="12" t="s">
+      <c r="G3" s="14" t="s">
         <v>52</v>
+      </c>
+      <c r="H3" s="15" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9" t="n">
+      <c r="A4" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="C4" s="11" t="n">
+      <c r="B4" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="C4" s="13" t="n">
         <v>33472</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="G4" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="G4" s="14" t="s">
         <v>44</v>
+      </c>
+      <c r="H4" s="15" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="n">
+      <c r="A5" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="C5" s="11" t="n">
+      <c r="B5" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" s="13" t="n">
         <v>36760</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="G5" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="G5" s="14" t="s">
         <v>52</v>
+      </c>
+      <c r="H5" s="15" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Alien validation consistency… (#331)
* Fix alien fields check for validate button, validate action and validate program.
Removed unused fail_if_alien checkbox from the import form
Fix/add unit tests

* Fix failing tests

* Fix failing tests
</commit_message>
<xml_diff>
--- a/tests/data/rdi_correct.xlsx
+++ b/tests/data/rdi_correct.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Households" sheetId="1" state="visible" r:id="rId3"/>
@@ -132,13 +132,13 @@
     <t xml:space="preserve">estimated_birth_date_i_c</t>
   </si>
   <si>
-    <t xml:space="preserve">national_id_no_i_c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">national_id_photo_i_c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">national_id_issuer_i_c</t>
+    <t xml:space="preserve">national_id_document_number_i_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">national_id_image_i_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">national_id_country_i_c</t>
   </si>
   <si>
     <t xml:space="preserve">phone_no_i_c</t>
@@ -343,14 +343,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
     <numFmt numFmtId="166" formatCode="@"/>
-    <numFmt numFmtId="167" formatCode="General"/>
-    <numFmt numFmtId="168" formatCode="m/d/yyyy"/>
-    <numFmt numFmtId="169" formatCode="0"/>
-    <numFmt numFmtId="170" formatCode="d/m/yyyy\ hh:mm:ss"/>
+    <numFmt numFmtId="167" formatCode="m/d/yyyy"/>
+    <numFmt numFmtId="168" formatCode="0"/>
+    <numFmt numFmtId="169" formatCode="d/m/yyyy\ hh:mm:ss"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -451,7 +450,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -480,11 +479,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -496,7 +495,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -504,16 +503,12 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="169" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -556,13 +551,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>96120</xdr:colOff>
+      <xdr:colOff>95760</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>93240</xdr:rowOff>
+      <xdr:rowOff>92880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="Image 3" descr=""/>
+        <xdr:cNvPr id="1" name="Image 3"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -572,11 +567,12 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="17452440" y="380880"/>
-          <a:ext cx="96120" cy="93240"/>
+          <a:ext cx="95760" cy="92880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:noFill/>
         <a:ln w="0">
           <a:noFill/>
         </a:ln>
@@ -593,13 +589,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>96480</xdr:colOff>
+      <xdr:colOff>96120</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>93600</xdr:rowOff>
+      <xdr:rowOff>93240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Image 1" descr=""/>
+        <xdr:cNvPr id="2" name="Image 1"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -609,11 +605,12 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10877400" y="380880"/>
-          <a:ext cx="96480" cy="93600"/>
+          <a:ext cx="96120" cy="93240"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:noFill/>
         <a:ln w="0">
           <a:noFill/>
         </a:ln>
@@ -805,7 +802,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:O4"/>
-  <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9.63"/>
@@ -938,7 +935,7 @@
       <c r="A4" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B4" s="7" t="b">
+      <c r="B4" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -996,7 +993,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:P13"/>
-  <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.82"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.97"/>
@@ -1050,7 +1047,7 @@
       <c r="K1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="7" t="s">
         <v>35</v>
       </c>
       <c r="M1" s="2" t="s">
@@ -1327,7 +1324,7 @@
       <c r="J8" s="8" t="n">
         <v>25778</v>
       </c>
-      <c r="K8" s="7" t="b">
+      <c r="K8" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1369,7 +1366,7 @@
       <c r="J9" s="8" t="n">
         <v>31934</v>
       </c>
-      <c r="K9" s="7" t="b">
+      <c r="K9" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1411,7 +1408,7 @@
       <c r="J10" s="8" t="n">
         <v>23346</v>
       </c>
-      <c r="K10" s="7" t="b">
+      <c r="K10" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1460,7 +1457,7 @@
       <c r="J13" s="8" t="n">
         <v>42889</v>
       </c>
-      <c r="K13" s="7" t="b">
+      <c r="K13" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1493,7 +1490,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30.18"/>
@@ -1553,7 +1550,7 @@
       <c r="G2" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="H2" s="15" t="b">
+      <c r="H2" s="10" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1580,7 +1577,7 @@
       <c r="G3" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="H3" s="15" t="b">
+      <c r="H3" s="10" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1607,7 +1604,7 @@
       <c r="G4" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="H4" s="15" t="b">
+      <c r="H4" s="10" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1634,7 +1631,7 @@
       <c r="G5" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="H5" s="15" t="b">
+      <c r="H5" s="10" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>

</xml_diff>